<commit_message>
Final results, recommendation and README case study
</commit_message>
<xml_diff>
--- a/roi/roi_model.xlsx
+++ b/roi/roi_model.xlsx
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="273">
   <si>
     <t xml:space="preserve">AI Customer Support Assistant: ROI Model</t>
   </si>
   <si>
-    <t xml:space="preserve">Harbor &amp; Thread (fictional) | Step 9 of 11 | Author: Mohammed Omer Ahmed | Version 1.0 (draft)</t>
+    <t xml:space="preserve">Harbor &amp; Thread (fictional) | Step 9 of 11 | Author: Mohammed Omer Ahmed | Version 1.1 (prototype results added)</t>
   </si>
   <si>
     <t xml:space="preserve">What it answers</t>
@@ -129,7 +129,7 @@
     <t xml:space="preserve">Containment</t>
   </si>
   <si>
-    <t xml:space="preserve">The expected containment rate (60%) is the pilot target from the test plan. Step 10 replaces it with the prototype's measured results.</t>
+    <t xml:space="preserve">The expected containment rate (60%) is the pilot target from the test plan. The prototype can't measure real containment, but its routing test shows 88.4% of tier A and B chats reach the AI, which caps containment. Every scenario stays below that cap (Inputs, row 36).</t>
   </si>
   <si>
     <t xml:space="preserve">Staffing</t>
@@ -394,6 +394,21 @@
   </si>
   <si>
     <t xml:space="preserve">Example of the expected format: 0.60 shows as 60.0%. Enter percentages as decimals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prototype result (Step 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of tier A and B chats routed to the AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-36, final run on 521 real ABCD conversations: 153 of 173 tier A and B chats reached the AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check: containment in every scenario is at or below that share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The AI can only resolve chats that reach it, so routing sets a ceiling on containment</t>
   </si>
   <si>
     <t xml:space="preserve">Model: calculations by scenario</t>
@@ -1159,6 +1174,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1180,10 +1203,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1212,10 +1231,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1534,11 +1549,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="42675350"/>
-        <c:axId val="20248484"/>
+        <c:axId val="18206117"/>
+        <c:axId val="69013449"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="42675350"/>
+        <c:axId val="18206117"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1570,7 +1585,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20248484"/>
+        <c:crossAx val="69013449"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1578,7 +1593,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="20248484"/>
+        <c:axId val="69013449"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1654,7 +1669,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42675350"/>
+        <c:crossAx val="18206117"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2081,7 +2096,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="3" t="s">
         <v>33</v>
       </c>
@@ -2463,7 +2478,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -2842,6 +2857,43 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
         <v>122</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C34" s="10"/>
+      <c r="E34" s="10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="B35" s="32" t="n">
+        <v>0.884393063583815</v>
+      </c>
+      <c r="C35" s="11"/>
+      <c r="E35" s="20" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B36" s="33" t="str">
+        <f aca="false">IF(MAX(B23:D23)&lt;=B35,"OK","Too high: containment can't exceed routing")</f>
+        <v>OK</v>
+      </c>
+      <c r="C36" s="11"/>
+      <c r="E36" s="20" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -2870,17 +2922,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>57</v>
@@ -2892,853 +2944,853 @@
         <v>59</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="32" t="s">
-        <v>127</v>
-      </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
+      <c r="A6" s="34" t="s">
+        <v>132</v>
+      </c>
+      <c r="B6" s="35"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="B7" s="35" t="n">
+      <c r="A7" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$6/60</f>
         <v>4000</v>
       </c>
-      <c r="C7" s="35" t="n">
+      <c r="C7" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$6/60</f>
         <v>4000</v>
       </c>
-      <c r="D7" s="35" t="n">
+      <c r="D7" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$6/60</f>
         <v>4000</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="B8" s="36" t="n">
+      <c r="A8" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="B8" s="38" t="n">
         <f aca="false">B7*Inputs!$B$7</f>
         <v>128000</v>
       </c>
-      <c r="C8" s="36" t="n">
+      <c r="C8" s="38" t="n">
         <f aca="false">C7*Inputs!$B$7</f>
         <v>128000</v>
       </c>
-      <c r="D8" s="36" t="n">
+      <c r="D8" s="38" t="n">
         <f aca="false">D7*Inputs!$B$7</f>
         <v>128000</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="B9" s="35" t="n">
+      <c r="A9" s="36" t="s">
+        <v>137</v>
+      </c>
+      <c r="B9" s="37" t="n">
         <f aca="false">Inputs!$B$8*Inputs!$B$9</f>
         <v>5600</v>
       </c>
-      <c r="C9" s="35" t="n">
+      <c r="C9" s="37" t="n">
         <f aca="false">Inputs!$B$8*Inputs!$B$9</f>
         <v>5600</v>
       </c>
-      <c r="D9" s="35" t="n">
+      <c r="D9" s="37" t="n">
         <f aca="false">Inputs!$B$8*Inputs!$B$9</f>
         <v>5600</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="34" t="s">
-        <v>134</v>
-      </c>
-      <c r="B10" s="37" t="n">
+      <c r="A10" s="36" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="39" t="n">
         <f aca="false">IF(B9&gt;0,B7/B9,0)</f>
         <v>0.714285714285714</v>
       </c>
-      <c r="C10" s="37" t="n">
+      <c r="C10" s="39" t="n">
         <f aca="false">IF(C9&gt;0,C7/C9,0)</f>
         <v>0.714285714285714</v>
       </c>
-      <c r="D10" s="37" t="n">
+      <c r="D10" s="39" t="n">
         <f aca="false">IF(D9&gt;0,D7/D9,0)</f>
         <v>0.714285714285714</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="32" t="s">
-        <v>136</v>
-      </c>
-      <c r="B12" s="33"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
-      <c r="E12" s="33"/>
+      <c r="A12" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="B13" s="35" t="n">
+      <c r="A13" s="36" t="s">
+        <v>142</v>
+      </c>
+      <c r="B13" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$16</f>
         <v>9455.28779127664</v>
       </c>
-      <c r="C13" s="35" t="n">
+      <c r="C13" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$16</f>
         <v>9455.28779127664</v>
       </c>
-      <c r="D13" s="35" t="n">
+      <c r="D13" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$16</f>
         <v>9455.28779127664</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34" t="s">
-        <v>139</v>
-      </c>
-      <c r="B14" s="35" t="n">
+      <c r="A14" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="B14" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$17</f>
         <v>3587.93069109739</v>
       </c>
-      <c r="C14" s="35" t="n">
+      <c r="C14" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$17</f>
         <v>3587.93069109739</v>
       </c>
-      <c r="D14" s="35" t="n">
+      <c r="D14" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$17</f>
         <v>3587.93069109739</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34" t="s">
-        <v>140</v>
-      </c>
-      <c r="B15" s="35" t="n">
+      <c r="A15" s="36" t="s">
+        <v>145</v>
+      </c>
+      <c r="B15" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$18</f>
         <v>13264.2899820753</v>
       </c>
-      <c r="C15" s="35" t="n">
+      <c r="C15" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$18</f>
         <v>13264.2899820753</v>
       </c>
-      <c r="D15" s="35" t="n">
+      <c r="D15" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$18</f>
         <v>13264.2899820753</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34" t="s">
-        <v>141</v>
-      </c>
-      <c r="B16" s="35" t="n">
+      <c r="A16" s="36" t="s">
+        <v>146</v>
+      </c>
+      <c r="B16" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$19</f>
         <v>3692.49153555069</v>
       </c>
-      <c r="C16" s="35" t="n">
+      <c r="C16" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$19</f>
         <v>3692.49153555069</v>
       </c>
-      <c r="D16" s="35" t="n">
+      <c r="D16" s="37" t="n">
         <f aca="false">Inputs!$B$5*Inputs!$B$19</f>
         <v>3692.49153555069</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="32" t="s">
-        <v>142</v>
-      </c>
-      <c r="B18" s="33"/>
-      <c r="C18" s="33"/>
-      <c r="D18" s="33"/>
-      <c r="E18" s="33"/>
+      <c r="A18" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="B19" s="35" t="n">
+      <c r="A19" s="36" t="s">
+        <v>148</v>
+      </c>
+      <c r="B19" s="37" t="n">
         <f aca="false">(B13+B14)*Inputs!B23</f>
         <v>5217.28739294961</v>
       </c>
-      <c r="C19" s="35" t="n">
+      <c r="C19" s="37" t="n">
         <f aca="false">(C13+C14)*Inputs!C23</f>
         <v>7825.93108942442</v>
       </c>
-      <c r="D19" s="35" t="n">
+      <c r="D19" s="37" t="n">
         <f aca="false">(D13+D14)*Inputs!D23</f>
         <v>9782.41386178052</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="B20" s="35" t="n">
+      <c r="A20" s="36" t="s">
+        <v>150</v>
+      </c>
+      <c r="B20" s="37" t="n">
         <f aca="false">B19*Inputs!$B$6/60</f>
         <v>695.638319059948</v>
       </c>
-      <c r="C20" s="35" t="n">
+      <c r="C20" s="37" t="n">
         <f aca="false">C19*Inputs!$B$6/60</f>
         <v>1043.45747858992</v>
       </c>
-      <c r="D20" s="35" t="n">
+      <c r="D20" s="37" t="n">
         <f aca="false">D19*Inputs!$B$6/60</f>
         <v>1304.3218482374</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="38" t="s">
-        <v>147</v>
-      </c>
-      <c r="B21" s="39" t="n">
+      <c r="A21" s="33" t="s">
+        <v>152</v>
+      </c>
+      <c r="B21" s="40" t="n">
         <f aca="false">B20*Inputs!$B$7</f>
         <v>22260.4262099183</v>
       </c>
-      <c r="C21" s="39" t="n">
+      <c r="C21" s="40" t="n">
         <f aca="false">C20*Inputs!$B$7</f>
         <v>33390.6393148775</v>
       </c>
-      <c r="D21" s="39" t="n">
+      <c r="D21" s="40" t="n">
         <f aca="false">D20*Inputs!$B$7</f>
         <v>41738.2991435969</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="34" t="s">
-        <v>149</v>
-      </c>
-      <c r="B22" s="36" t="n">
+      <c r="A22" s="36" t="s">
+        <v>154</v>
+      </c>
+      <c r="B22" s="38" t="n">
         <f aca="false">Inputs!$B$5*Inputs!B26</f>
         <v>6000</v>
       </c>
-      <c r="C22" s="36" t="n">
+      <c r="C22" s="38" t="n">
         <f aca="false">Inputs!$B$5*Inputs!C26</f>
         <v>3000</v>
       </c>
-      <c r="D22" s="36" t="n">
+      <c r="D22" s="38" t="n">
         <f aca="false">Inputs!$B$5*Inputs!D26</f>
         <v>1500</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="34" t="s">
-        <v>151</v>
-      </c>
-      <c r="B23" s="36" t="n">
+      <c r="A23" s="36" t="s">
+        <v>156</v>
+      </c>
+      <c r="B23" s="38" t="n">
         <f aca="false">B19*Inputs!B27</f>
         <v>7825.93108942442</v>
       </c>
-      <c r="C23" s="36" t="n">
+      <c r="C23" s="38" t="n">
         <f aca="false">C19*Inputs!C27</f>
         <v>7747.67177853017</v>
       </c>
-      <c r="D23" s="36" t="n">
+      <c r="D23" s="38" t="n">
         <f aca="false">D19*Inputs!D27</f>
         <v>7336.81039633539</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="34" t="s">
-        <v>153</v>
-      </c>
-      <c r="B24" s="36" t="n">
+      <c r="A24" s="36" t="s">
+        <v>158</v>
+      </c>
+      <c r="B24" s="38" t="n">
         <f aca="false">Inputs!B28</f>
         <v>4000</v>
       </c>
-      <c r="C24" s="36" t="n">
+      <c r="C24" s="38" t="n">
         <f aca="false">Inputs!C28</f>
         <v>2500</v>
       </c>
-      <c r="D24" s="36" t="n">
+      <c r="D24" s="38" t="n">
         <f aca="false">Inputs!D28</f>
         <v>2000</v>
       </c>
       <c r="E24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="34" t="s">
-        <v>154</v>
-      </c>
-      <c r="B25" s="36" t="n">
+      <c r="A25" s="36" t="s">
+        <v>159</v>
+      </c>
+      <c r="B25" s="38" t="n">
         <f aca="false">Inputs!$B$10*Inputs!$B$12*Inputs!$B$11</f>
         <v>1039.2</v>
       </c>
-      <c r="C25" s="36" t="n">
+      <c r="C25" s="38" t="n">
         <f aca="false">Inputs!$B$10*Inputs!$B$12*Inputs!$B$11</f>
         <v>1039.2</v>
       </c>
-      <c r="D25" s="36" t="n">
+      <c r="D25" s="38" t="n">
         <f aca="false">Inputs!$B$10*Inputs!$B$12*Inputs!$B$11</f>
         <v>1039.2</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="38" t="s">
-        <v>156</v>
-      </c>
-      <c r="B26" s="39" t="n">
+      <c r="A26" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="B26" s="40" t="n">
         <f aca="false">SUM(B22:B25)</f>
         <v>18865.1310894244</v>
       </c>
-      <c r="C26" s="39" t="n">
+      <c r="C26" s="40" t="n">
         <f aca="false">SUM(C22:C25)</f>
         <v>14286.8717785302</v>
       </c>
-      <c r="D26" s="39" t="n">
+      <c r="D26" s="40" t="n">
         <f aca="false">SUM(D22:D25)</f>
         <v>11876.0103963354</v>
       </c>
       <c r="E26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="38" t="s">
-        <v>157</v>
-      </c>
-      <c r="B27" s="39" t="n">
+      <c r="A27" s="33" t="s">
+        <v>162</v>
+      </c>
+      <c r="B27" s="40" t="n">
         <f aca="false">B21-B26</f>
         <v>3395.29512049392</v>
       </c>
-      <c r="C27" s="39" t="n">
+      <c r="C27" s="40" t="n">
         <f aca="false">C21-C26</f>
         <v>19103.7675363473</v>
       </c>
-      <c r="D27" s="39" t="n">
+      <c r="D27" s="40" t="n">
         <f aca="false">D21-D26</f>
         <v>29862.2887472615</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="B28" s="39" t="n">
+      <c r="A28" s="33" t="s">
+        <v>164</v>
+      </c>
+      <c r="B28" s="40" t="n">
         <f aca="false">B27*12</f>
         <v>40743.5414459271</v>
       </c>
-      <c r="C28" s="39" t="n">
+      <c r="C28" s="40" t="n">
         <f aca="false">C27*12</f>
         <v>229245.210436168</v>
       </c>
-      <c r="D28" s="39" t="n">
+      <c r="D28" s="40" t="n">
         <f aca="false">D27*12</f>
         <v>358347.464967138</v>
       </c>
       <c r="E28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="34" t="s">
-        <v>160</v>
-      </c>
-      <c r="B29" s="36" t="n">
+      <c r="A29" s="36" t="s">
+        <v>165</v>
+      </c>
+      <c r="B29" s="38" t="n">
         <f aca="false">Inputs!B29</f>
         <v>160000</v>
       </c>
-      <c r="C29" s="36" t="n">
+      <c r="C29" s="38" t="n">
         <f aca="false">Inputs!C29</f>
         <v>120000</v>
       </c>
-      <c r="D29" s="36" t="n">
+      <c r="D29" s="38" t="n">
         <f aca="false">Inputs!D29</f>
         <v>90000</v>
       </c>
       <c r="E29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="34" t="s">
-        <v>161</v>
-      </c>
-      <c r="B30" s="40" t="n">
+      <c r="A30" s="36" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="41" t="n">
         <f aca="false">IF(B27&gt;0,B29/B27,"No payback")</f>
         <v>47.1240332053151</v>
       </c>
-      <c r="C30" s="40" t="n">
+      <c r="C30" s="41" t="n">
         <f aca="false">IF(C27&gt;0,C29/C27,"No payback")</f>
         <v>6.28148347029898</v>
       </c>
-      <c r="D30" s="40" t="n">
+      <c r="D30" s="41" t="n">
         <f aca="false">IF(D27&gt;0,D29/D27,"No payback")</f>
         <v>3.01383463142132</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="34" t="s">
-        <v>163</v>
-      </c>
-      <c r="B31" s="36" t="n">
+      <c r="A31" s="36" t="s">
+        <v>168</v>
+      </c>
+      <c r="B31" s="38" t="n">
         <f aca="false">B27*Inputs!$B$13-B29</f>
         <v>-37769.3756622188</v>
       </c>
-      <c r="C31" s="36" t="n">
+      <c r="C31" s="38" t="n">
         <f aca="false">C27*Inputs!$B$13-C29</f>
         <v>567735.631308504</v>
       </c>
-      <c r="D31" s="36" t="n">
+      <c r="D31" s="38" t="n">
         <f aca="false">D27*Inputs!$B$13-D29</f>
         <v>985042.394901414</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="34" t="s">
-        <v>165</v>
-      </c>
-      <c r="B32" s="37" t="n">
+      <c r="A32" s="36" t="s">
+        <v>170</v>
+      </c>
+      <c r="B32" s="39" t="n">
         <f aca="false">IF(B29&gt;0,B31/B29,0)</f>
         <v>-0.236058597888867</v>
       </c>
-      <c r="C32" s="37" t="n">
+      <c r="C32" s="39" t="n">
         <f aca="false">IF(C29&gt;0,C31/C29,0)</f>
         <v>4.7311302609042</v>
       </c>
-      <c r="D32" s="37" t="n">
+      <c r="D32" s="39" t="n">
         <f aca="false">IF(D29&gt;0,D31/D29,0)</f>
         <v>10.9449154989046</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="34" t="s">
-        <v>167</v>
-      </c>
-      <c r="B33" s="41" t="n">
+      <c r="A33" s="36" t="s">
+        <v>172</v>
+      </c>
+      <c r="B33" s="42" t="n">
         <f aca="false">IF(Inputs!$B$9&gt;0,B20/Inputs!$B$9,0)</f>
         <v>4.96884513614249</v>
       </c>
-      <c r="C33" s="41" t="n">
+      <c r="C33" s="42" t="n">
         <f aca="false">IF(Inputs!$B$9&gt;0,C20/Inputs!$B$9,0)</f>
         <v>7.45326770421373</v>
       </c>
-      <c r="D33" s="41" t="n">
+      <c r="D33" s="42" t="n">
         <f aca="false">IF(Inputs!$B$9&gt;0,D20/Inputs!$B$9,0)</f>
         <v>9.31658463026716</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="B34" s="42" t="n">
+      <c r="A34" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="B34" s="43" t="n">
         <f aca="false">(B22+B24+B25)/((B13+B14)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!B27))</f>
         <v>0.305911634812268</v>
       </c>
-      <c r="C34" s="42" t="n">
+      <c r="C34" s="43" t="n">
         <f aca="false">(C22+C24+C25)/((C13+C14)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!C27))</f>
         <v>0.153005692279517</v>
       </c>
-      <c r="D34" s="42" t="n">
+      <c r="D34" s="43" t="n">
         <f aca="false">(D22+D24+D25)/((D13+D14)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!D27))</f>
         <v>0.098960833497969</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="38" t="s">
-        <v>171</v>
-      </c>
-      <c r="B35" s="42" t="n">
+      <c r="A35" s="33" t="s">
+        <v>176</v>
+      </c>
+      <c r="B35" s="43" t="n">
         <f aca="false">(B22+B24+B25+B29/12)/((B13+B14)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!B27))</f>
         <v>0.67539690525731</v>
       </c>
-      <c r="C35" s="42" t="n">
+      <c r="C35" s="43" t="n">
         <f aca="false">(C22+C24+C25+C29/12)/((C13+C14)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!C27))</f>
         <v>0.386987971884846</v>
       </c>
-      <c r="D35" s="42" t="n">
+      <c r="D35" s="43" t="n">
         <f aca="false">(D22+D24+D25+D29/12)/((D13+D14)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!D27))</f>
         <v>0.262471199032594</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="32" t="s">
-        <v>173</v>
-      </c>
-      <c r="B37" s="33"/>
-      <c r="C37" s="33"/>
-      <c r="D37" s="33"/>
-      <c r="E37" s="33"/>
+      <c r="A37" s="34" t="s">
+        <v>178</v>
+      </c>
+      <c r="B37" s="35"/>
+      <c r="C37" s="35"/>
+      <c r="D37" s="35"/>
+      <c r="E37" s="35"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="34" t="s">
-        <v>174</v>
-      </c>
-      <c r="B38" s="35" t="n">
+      <c r="A38" s="36" t="s">
+        <v>179</v>
+      </c>
+      <c r="B38" s="37" t="n">
         <f aca="false">B15*Inputs!B24</f>
         <v>6632.14499103764</v>
       </c>
-      <c r="C38" s="35" t="n">
+      <c r="C38" s="37" t="n">
         <f aca="false">C15*Inputs!C24</f>
         <v>9285.0029874527</v>
       </c>
-      <c r="D38" s="35" t="n">
+      <c r="D38" s="37" t="n">
         <f aca="false">D15*Inputs!D24</f>
         <v>11274.646484764</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="34" t="s">
-        <v>176</v>
-      </c>
-      <c r="B39" s="35" t="n">
+      <c r="A39" s="36" t="s">
+        <v>181</v>
+      </c>
+      <c r="B39" s="37" t="n">
         <f aca="false">B38*(Inputs!$B$6-Inputs!B25)/60</f>
         <v>442.142999402509</v>
       </c>
-      <c r="C39" s="35" t="n">
+      <c r="C39" s="37" t="n">
         <f aca="false">C38*(Inputs!$B$6-Inputs!C25)/60</f>
         <v>928.50029874527</v>
       </c>
-      <c r="D39" s="35" t="n">
+      <c r="D39" s="37" t="n">
         <f aca="false">D38*(Inputs!$B$6-Inputs!D25)/60</f>
         <v>1221.42003584943</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="34" t="s">
-        <v>178</v>
-      </c>
-      <c r="B40" s="35" t="n">
+      <c r="A40" s="36" t="s">
+        <v>183</v>
+      </c>
+      <c r="B40" s="37" t="n">
         <f aca="false">B20+B39</f>
         <v>1137.78131846246</v>
       </c>
-      <c r="C40" s="35" t="n">
+      <c r="C40" s="37" t="n">
         <f aca="false">C20+C39</f>
         <v>1971.95777733519</v>
       </c>
-      <c r="D40" s="35" t="n">
+      <c r="D40" s="37" t="n">
         <f aca="false">D20+D39</f>
         <v>2525.74188408684</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="38" t="s">
-        <v>147</v>
-      </c>
-      <c r="B41" s="39" t="n">
+      <c r="A41" s="33" t="s">
+        <v>152</v>
+      </c>
+      <c r="B41" s="40" t="n">
         <f aca="false">B40*Inputs!$B$7</f>
         <v>36409.0021907986</v>
       </c>
-      <c r="C41" s="39" t="n">
+      <c r="C41" s="40" t="n">
         <f aca="false">C40*Inputs!$B$7</f>
         <v>63102.6488747262</v>
       </c>
-      <c r="D41" s="39" t="n">
+      <c r="D41" s="40" t="n">
         <f aca="false">D40*Inputs!$B$7</f>
         <v>80823.7402907787</v>
       </c>
       <c r="E41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="34" t="s">
-        <v>149</v>
-      </c>
-      <c r="B42" s="36" t="n">
+      <c r="A42" s="36" t="s">
+        <v>154</v>
+      </c>
+      <c r="B42" s="38" t="n">
         <f aca="false">B22</f>
         <v>6000</v>
       </c>
-      <c r="C42" s="36" t="n">
+      <c r="C42" s="38" t="n">
         <f aca="false">C22</f>
         <v>3000</v>
       </c>
-      <c r="D42" s="36" t="n">
+      <c r="D42" s="38" t="n">
         <f aca="false">D22</f>
         <v>1500</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="34" t="s">
-        <v>151</v>
-      </c>
-      <c r="B43" s="36" t="n">
+      <c r="A43" s="36" t="s">
+        <v>156</v>
+      </c>
+      <c r="B43" s="38" t="n">
         <f aca="false">(B19+B38)*Inputs!B27</f>
         <v>17774.1485759809</v>
       </c>
-      <c r="C43" s="36" t="n">
+      <c r="C43" s="38" t="n">
         <f aca="false">(C19+C38)*Inputs!C27</f>
         <v>16939.8247361083</v>
       </c>
-      <c r="D43" s="36" t="n">
+      <c r="D43" s="38" t="n">
         <f aca="false">(D19+D38)*Inputs!D27</f>
         <v>15792.7952599084</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="34" t="s">
-        <v>153</v>
-      </c>
-      <c r="B44" s="36" t="n">
+      <c r="A44" s="36" t="s">
+        <v>158</v>
+      </c>
+      <c r="B44" s="38" t="n">
         <f aca="false">B24</f>
         <v>4000</v>
       </c>
-      <c r="C44" s="36" t="n">
+      <c r="C44" s="38" t="n">
         <f aca="false">C24</f>
         <v>2500</v>
       </c>
-      <c r="D44" s="36" t="n">
+      <c r="D44" s="38" t="n">
         <f aca="false">D24</f>
         <v>2000</v>
       </c>
       <c r="E44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="34" t="s">
-        <v>154</v>
-      </c>
-      <c r="B45" s="36" t="n">
+      <c r="A45" s="36" t="s">
+        <v>159</v>
+      </c>
+      <c r="B45" s="38" t="n">
         <f aca="false">B25</f>
         <v>1039.2</v>
       </c>
-      <c r="C45" s="36" t="n">
+      <c r="C45" s="38" t="n">
         <f aca="false">C25</f>
         <v>1039.2</v>
       </c>
-      <c r="D45" s="36" t="n">
+      <c r="D45" s="38" t="n">
         <f aca="false">D25</f>
         <v>1039.2</v>
       </c>
       <c r="E45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="38" t="s">
-        <v>156</v>
-      </c>
-      <c r="B46" s="39" t="n">
+      <c r="A46" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="B46" s="40" t="n">
         <f aca="false">SUM(B42:B45)</f>
         <v>28813.3485759809</v>
       </c>
-      <c r="C46" s="39" t="n">
+      <c r="C46" s="40" t="n">
         <f aca="false">SUM(C42:C45)</f>
         <v>23479.0247361083</v>
       </c>
-      <c r="D46" s="39" t="n">
+      <c r="D46" s="40" t="n">
         <f aca="false">SUM(D42:D45)</f>
         <v>20331.9952599084</v>
       </c>
       <c r="E46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="38" t="s">
-        <v>157</v>
-      </c>
-      <c r="B47" s="39" t="n">
+      <c r="A47" s="33" t="s">
+        <v>162</v>
+      </c>
+      <c r="B47" s="40" t="n">
         <f aca="false">B41-B46</f>
         <v>7595.65361481777</v>
       </c>
-      <c r="C47" s="39" t="n">
+      <c r="C47" s="40" t="n">
         <f aca="false">C41-C46</f>
         <v>39623.6241386178</v>
       </c>
-      <c r="D47" s="39" t="n">
+      <c r="D47" s="40" t="n">
         <f aca="false">D41-D46</f>
         <v>60491.7450308703</v>
       </c>
       <c r="E47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="B48" s="39" t="n">
+      <c r="A48" s="33" t="s">
+        <v>164</v>
+      </c>
+      <c r="B48" s="40" t="n">
         <f aca="false">B47*12</f>
         <v>91147.8433778132</v>
       </c>
-      <c r="C48" s="39" t="n">
+      <c r="C48" s="40" t="n">
         <f aca="false">C47*12</f>
         <v>475483.489663414</v>
       </c>
-      <c r="D48" s="39" t="n">
+      <c r="D48" s="40" t="n">
         <f aca="false">D47*12</f>
         <v>725900.940370444</v>
       </c>
       <c r="E48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="34" t="s">
-        <v>182</v>
-      </c>
-      <c r="B49" s="36" t="n">
+      <c r="A49" s="36" t="s">
+        <v>187</v>
+      </c>
+      <c r="B49" s="38" t="n">
         <f aca="false">Inputs!B29+Inputs!B30</f>
         <v>270000</v>
       </c>
-      <c r="C49" s="36" t="n">
+      <c r="C49" s="38" t="n">
         <f aca="false">Inputs!C29+Inputs!C30</f>
         <v>200000</v>
       </c>
-      <c r="D49" s="36" t="n">
+      <c r="D49" s="38" t="n">
         <f aca="false">Inputs!D29+Inputs!D30</f>
         <v>150000</v>
       </c>
       <c r="E49" s="2"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="34" t="s">
-        <v>161</v>
-      </c>
-      <c r="B50" s="40" t="n">
+      <c r="A50" s="36" t="s">
+        <v>166</v>
+      </c>
+      <c r="B50" s="41" t="n">
         <f aca="false">IF(B47&gt;0,B49/B47,"No payback")</f>
         <v>35.5466446591611</v>
       </c>
-      <c r="C50" s="40" t="n">
+      <c r="C50" s="41" t="n">
         <f aca="false">IF(C47&gt;0,C49/C47,"No payback")</f>
         <v>5.04749387134119</v>
       </c>
-      <c r="D50" s="40" t="n">
+      <c r="D50" s="41" t="n">
         <f aca="false">IF(D47&gt;0,D49/D47,"No payback")</f>
         <v>2.47967718443982</v>
       </c>
       <c r="E50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="34" t="s">
-        <v>163</v>
-      </c>
-      <c r="B51" s="36" t="n">
+      <c r="A51" s="36" t="s">
+        <v>168</v>
+      </c>
+      <c r="B51" s="38" t="n">
         <f aca="false">B47*Inputs!$B$13-B49</f>
         <v>3443.53013343958</v>
       </c>
-      <c r="C51" s="36" t="n">
+      <c r="C51" s="38" t="n">
         <f aca="false">C47*Inputs!$B$13-C49</f>
         <v>1226450.46899024</v>
       </c>
-      <c r="D51" s="36" t="n">
+      <c r="D51" s="38" t="n">
         <f aca="false">D47*Inputs!$B$13-D49</f>
         <v>2027702.82111133</v>
       </c>
       <c r="E51" s="2"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="34" t="s">
-        <v>165</v>
-      </c>
-      <c r="B52" s="37" t="n">
+      <c r="A52" s="36" t="s">
+        <v>170</v>
+      </c>
+      <c r="B52" s="39" t="n">
         <f aca="false">IF(B49&gt;0,B51/B49,0)</f>
         <v>0.0127538153090355</v>
       </c>
-      <c r="C52" s="37" t="n">
+      <c r="C52" s="39" t="n">
         <f aca="false">IF(C49&gt;0,C51/C49,0)</f>
         <v>6.1322523449512</v>
       </c>
-      <c r="D52" s="37" t="n">
+      <c r="D52" s="39" t="n">
         <f aca="false">IF(D49&gt;0,D51/D49,0)</f>
         <v>13.5180188074089</v>
       </c>
       <c r="E52" s="2"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="34" t="s">
-        <v>167</v>
-      </c>
-      <c r="B53" s="41" t="n">
+      <c r="A53" s="36" t="s">
+        <v>172</v>
+      </c>
+      <c r="B53" s="42" t="n">
         <f aca="false">IF(Inputs!$B$9&gt;0,B40/Inputs!$B$9,0)</f>
         <v>8.12700941758898</v>
       </c>
-      <c r="C53" s="41" t="n">
+      <c r="C53" s="42" t="n">
         <f aca="false">IF(Inputs!$B$9&gt;0,C40/Inputs!$B$9,0)</f>
         <v>14.0854126952514</v>
       </c>
-      <c r="D53" s="41" t="n">
+      <c r="D53" s="42" t="n">
         <f aca="false">IF(Inputs!$B$9&gt;0,D40/Inputs!$B$9,0)</f>
         <v>18.0410134577631</v>
       </c>
       <c r="E53" s="2"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="34" t="s">
-        <v>183</v>
-      </c>
-      <c r="B54" s="37" t="n">
+      <c r="A54" s="36" t="s">
+        <v>188</v>
+      </c>
+      <c r="B54" s="39" t="n">
         <f aca="false">IF(B7&gt;0,B40/B7,0)</f>
         <v>0.284445329615614</v>
       </c>
-      <c r="C54" s="37" t="n">
+      <c r="C54" s="39" t="n">
         <f aca="false">IF(C7&gt;0,C40/C7,0)</f>
         <v>0.492989444333798</v>
       </c>
-      <c r="D54" s="37" t="n">
+      <c r="D54" s="39" t="n">
         <f aca="false">IF(D7&gt;0,D40/D7,0)</f>
         <v>0.631435471021709</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -3767,228 +3819,228 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="27" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="43" t="s">
-        <v>188</v>
-      </c>
-      <c r="B5" s="44" t="n">
+      <c r="A5" s="44" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="45" t="n">
         <v>0.25</v>
       </c>
-      <c r="C5" s="44" t="n">
+      <c r="C5" s="45" t="n">
         <v>0.35</v>
       </c>
-      <c r="D5" s="45" t="n">
+      <c r="D5" s="46" t="n">
         <f aca="false">Inputs!$B$16+Inputs!$B$17</f>
         <v>0.434773949412468</v>
       </c>
-      <c r="E5" s="44" t="n">
+      <c r="E5" s="45" t="n">
         <v>0.55</v>
       </c>
-      <c r="F5" s="44" t="n">
+      <c r="F5" s="45" t="n">
         <v>0.65</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="46" t="n">
+      <c r="A6" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="B6" s="36" t="n">
+      <c r="B6" s="38" t="n">
         <f aca="false">$A6*(Inputs!$B$5*B$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>833.299999999999</v>
       </c>
-      <c r="C6" s="36" t="n">
+      <c r="C6" s="38" t="n">
         <f aca="false">$A6*(Inputs!$B$5*C$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>3782.3</v>
       </c>
-      <c r="D6" s="36" t="n">
+      <c r="D6" s="38" t="n">
         <f aca="false">$A6*(Inputs!$B$5*D$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>6282.28376817367</v>
       </c>
-      <c r="E6" s="36" t="n">
+      <c r="E6" s="38" t="n">
         <f aca="false">$A6*(Inputs!$B$5*E$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>9680.3</v>
       </c>
-      <c r="F6" s="36" t="n">
+      <c r="F6" s="38" t="n">
         <f aca="false">$A6*(Inputs!$B$5*F$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>12629.3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="46" t="n">
+      <c r="A7" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="B7" s="36" t="n">
+      <c r="B7" s="38" t="n">
         <f aca="false">$A7*(Inputs!$B$5*B$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>3290.8</v>
       </c>
-      <c r="C7" s="36" t="n">
+      <c r="C7" s="38" t="n">
         <f aca="false">$A7*(Inputs!$B$5*C$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>7222.8</v>
       </c>
-      <c r="D7" s="36" t="n">
+      <c r="D7" s="38" t="n">
         <f aca="false">$A7*(Inputs!$B$5*D$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>10556.1116908982</v>
       </c>
-      <c r="E7" s="36" t="n">
+      <c r="E7" s="38" t="n">
         <f aca="false">$A7*(Inputs!$B$5*E$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>15086.8</v>
       </c>
-      <c r="F7" s="36" t="n">
+      <c r="F7" s="38" t="n">
         <f aca="false">$A7*(Inputs!$B$5*F$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>19018.8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="46" t="n">
+      <c r="A8" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="B8" s="36" t="n">
+      <c r="B8" s="38" t="n">
         <f aca="false">$A8*(Inputs!$B$5*B$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>5748.3</v>
       </c>
-      <c r="C8" s="36" t="n">
+      <c r="C8" s="38" t="n">
         <f aca="false">$A8*(Inputs!$B$5*C$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>10663.3</v>
       </c>
-      <c r="D8" s="36" t="n">
+      <c r="D8" s="38" t="n">
         <f aca="false">$A8*(Inputs!$B$5*D$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>14829.9396136228</v>
       </c>
-      <c r="E8" s="36" t="n">
+      <c r="E8" s="38" t="n">
         <f aca="false">$A8*(Inputs!$B$5*E$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>20493.3</v>
       </c>
-      <c r="F8" s="36" t="n">
+      <c r="F8" s="38" t="n">
         <f aca="false">$A8*(Inputs!$B$5*F$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>25408.3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="46" t="n">
+      <c r="A9" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="B9" s="36" t="n">
+      <c r="B9" s="38" t="n">
         <f aca="false">$A9*(Inputs!$B$5*B$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>8205.8</v>
       </c>
-      <c r="C9" s="36" t="n">
+      <c r="C9" s="38" t="n">
         <f aca="false">$A9*(Inputs!$B$5*C$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>14103.8</v>
       </c>
-      <c r="D9" s="36" t="n">
+      <c r="D9" s="38" t="n">
         <f aca="false">$A9*(Inputs!$B$5*D$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>19103.7675363473</v>
       </c>
-      <c r="E9" s="36" t="n">
+      <c r="E9" s="38" t="n">
         <f aca="false">$A9*(Inputs!$B$5*E$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>25899.8</v>
       </c>
-      <c r="F9" s="36" t="n">
+      <c r="F9" s="38" t="n">
         <f aca="false">$A9*(Inputs!$B$5*F$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>31797.8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="46" t="n">
+      <c r="A10" s="32" t="n">
         <v>0.7</v>
       </c>
-      <c r="B10" s="36" t="n">
+      <c r="B10" s="38" t="n">
         <f aca="false">$A10*(Inputs!$B$5*B$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>10663.3</v>
       </c>
-      <c r="C10" s="36" t="n">
+      <c r="C10" s="38" t="n">
         <f aca="false">$A10*(Inputs!$B$5*C$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>17544.3</v>
       </c>
-      <c r="D10" s="36" t="n">
+      <c r="D10" s="38" t="n">
         <f aca="false">$A10*(Inputs!$B$5*D$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>23377.5954590719</v>
       </c>
-      <c r="E10" s="36" t="n">
+      <c r="E10" s="38" t="n">
         <f aca="false">$A10*(Inputs!$B$5*E$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>31306.3</v>
       </c>
-      <c r="F10" s="36" t="n">
+      <c r="F10" s="38" t="n">
         <f aca="false">$A10*(Inputs!$B$5*F$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>38187.3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="46" t="n">
+      <c r="A11" s="32" t="n">
         <v>0.8</v>
       </c>
-      <c r="B11" s="36" t="n">
+      <c r="B11" s="38" t="n">
         <f aca="false">$A11*(Inputs!$B$5*B$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>13120.8</v>
       </c>
-      <c r="C11" s="36" t="n">
+      <c r="C11" s="38" t="n">
         <f aca="false">$A11*(Inputs!$B$5*C$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>20984.8</v>
       </c>
-      <c r="D11" s="36" t="n">
+      <c r="D11" s="38" t="n">
         <f aca="false">$A11*(Inputs!$B$5*D$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>27651.4233817965</v>
       </c>
-      <c r="E11" s="36" t="n">
+      <c r="E11" s="38" t="n">
         <f aca="false">$A11*(Inputs!$B$5*E$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>36712.8</v>
       </c>
-      <c r="F11" s="36" t="n">
+      <c r="F11" s="38" t="n">
         <f aca="false">$A11*(Inputs!$B$5*F$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>44576.8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="46" t="n">
+      <c r="A12" s="32" t="n">
         <v>0.9</v>
       </c>
-      <c r="B12" s="36" t="n">
+      <c r="B12" s="38" t="n">
         <f aca="false">$A12*(Inputs!$B$5*B$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>15578.3</v>
       </c>
-      <c r="C12" s="36" t="n">
+      <c r="C12" s="38" t="n">
         <f aca="false">$A12*(Inputs!$B$5*C$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>24425.3</v>
       </c>
-      <c r="D12" s="36" t="n">
+      <c r="D12" s="38" t="n">
         <f aca="false">$A12*(Inputs!$B$5*D$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>31925.251304521</v>
       </c>
-      <c r="E12" s="36" t="n">
+      <c r="E12" s="38" t="n">
         <f aca="false">$A12*(Inputs!$B$5*E$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>42119.3</v>
       </c>
-      <c r="F12" s="36" t="n">
+      <c r="F12" s="38" t="n">
         <f aca="false">$A12*(Inputs!$B$5*F$5)*(Inputs!$B$6/60*Inputs!$B$7-Inputs!$C$27)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>50966.3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="43" t="s">
-        <v>191</v>
+      <c r="A17" s="44" t="s">
+        <v>196</v>
       </c>
       <c r="B17" s="47" t="n">
         <v>0.5</v>
@@ -4007,183 +4059,183 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="46" t="n">
+      <c r="A18" s="32" t="n">
         <v>0.3</v>
       </c>
-      <c r="B18" s="36" t="n">
+      <c r="B18" s="38" t="n">
         <f aca="false">$A18*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-B$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>8199.63688508265</v>
       </c>
-      <c r="C18" s="36" t="n">
+      <c r="C18" s="38" t="n">
         <f aca="false">$A18*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-C$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>7221.3954989046</v>
       </c>
-      <c r="D18" s="36" t="n">
+      <c r="D18" s="38" t="n">
         <f aca="false">$A18*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-D$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>6282.28376817367</v>
       </c>
-      <c r="E18" s="36" t="n">
+      <c r="E18" s="38" t="n">
         <f aca="false">$A18*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-E$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>5264.91272654849</v>
       </c>
-      <c r="F18" s="36" t="n">
+      <c r="F18" s="38" t="n">
         <f aca="false">$A18*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-F$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>4286.67134037044</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="46" t="n">
+      <c r="A19" s="32" t="n">
         <v>0.4</v>
       </c>
-      <c r="B19" s="36" t="n">
+      <c r="B19" s="38" t="n">
         <f aca="false">$A19*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-B$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>13112.5825134435</v>
       </c>
-      <c r="C19" s="36" t="n">
+      <c r="C19" s="38" t="n">
         <f aca="false">$A19*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-C$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>11808.2606652061</v>
       </c>
-      <c r="D19" s="36" t="n">
+      <c r="D19" s="38" t="n">
         <f aca="false">$A19*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-D$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>10556.1116908982</v>
       </c>
-      <c r="E19" s="36" t="n">
+      <c r="E19" s="38" t="n">
         <f aca="false">$A19*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-E$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>9199.61696873133</v>
       </c>
-      <c r="F19" s="36" t="n">
+      <c r="F19" s="38" t="n">
         <f aca="false">$A19*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-F$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>7895.29512049393</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="46" t="n">
+      <c r="A20" s="32" t="n">
         <v>0.5</v>
       </c>
-      <c r="B20" s="36" t="n">
+      <c r="B20" s="38" t="n">
         <f aca="false">$A20*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-B$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>18025.5281418044</v>
       </c>
-      <c r="C20" s="36" t="n">
+      <c r="C20" s="38" t="n">
         <f aca="false">$A20*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-C$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>16395.1258315077</v>
       </c>
-      <c r="D20" s="36" t="n">
+      <c r="D20" s="38" t="n">
         <f aca="false">$A20*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-D$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>14829.9396136228</v>
       </c>
-      <c r="E20" s="36" t="n">
+      <c r="E20" s="38" t="n">
         <f aca="false">$A20*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-E$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>13134.3212109142</v>
       </c>
-      <c r="F20" s="36" t="n">
+      <c r="F20" s="38" t="n">
         <f aca="false">$A20*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-F$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>11503.9189006174</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="46" t="n">
+      <c r="A21" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="B21" s="36" t="n">
+      <c r="B21" s="38" t="n">
         <f aca="false">$A21*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-B$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>22938.4737701653</v>
       </c>
-      <c r="C21" s="36" t="n">
+      <c r="C21" s="38" t="n">
         <f aca="false">$A21*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-C$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>20981.9909978092</v>
       </c>
-      <c r="D21" s="36" t="n">
+      <c r="D21" s="38" t="n">
         <f aca="false">$A21*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-D$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>19103.7675363473</v>
       </c>
-      <c r="E21" s="36" t="n">
+      <c r="E21" s="38" t="n">
         <f aca="false">$A21*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-E$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>17069.025453097</v>
       </c>
-      <c r="F21" s="36" t="n">
+      <c r="F21" s="38" t="n">
         <f aca="false">$A21*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-F$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>15112.5426807409</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="46" t="n">
+      <c r="A22" s="32" t="n">
         <v>0.7</v>
       </c>
-      <c r="B22" s="36" t="n">
+      <c r="B22" s="38" t="n">
         <f aca="false">$A22*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-B$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>27851.4193985262</v>
       </c>
-      <c r="C22" s="36" t="n">
+      <c r="C22" s="38" t="n">
         <f aca="false">$A22*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-C$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>25568.8561641107</v>
       </c>
-      <c r="D22" s="36" t="n">
+      <c r="D22" s="38" t="n">
         <f aca="false">$A22*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-D$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>23377.5954590719</v>
       </c>
-      <c r="E22" s="36" t="n">
+      <c r="E22" s="38" t="n">
         <f aca="false">$A22*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-E$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>21003.7296952798</v>
       </c>
-      <c r="F22" s="36" t="n">
+      <c r="F22" s="38" t="n">
         <f aca="false">$A22*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-F$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>18721.1664608644</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="46" t="n">
+      <c r="A23" s="32" t="n">
         <v>0.8</v>
       </c>
-      <c r="B23" s="36" t="n">
+      <c r="B23" s="38" t="n">
         <f aca="false">$A23*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-B$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>32764.3650268871</v>
       </c>
-      <c r="C23" s="36" t="n">
+      <c r="C23" s="38" t="n">
         <f aca="false">$A23*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-C$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>30155.7213304123</v>
       </c>
-      <c r="D23" s="36" t="n">
+      <c r="D23" s="38" t="n">
         <f aca="false">$A23*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-D$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>27651.4233817965</v>
       </c>
-      <c r="E23" s="36" t="n">
+      <c r="E23" s="38" t="n">
         <f aca="false">$A23*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-E$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>24938.4339374627</v>
       </c>
-      <c r="F23" s="36" t="n">
+      <c r="F23" s="38" t="n">
         <f aca="false">$A23*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-F$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>22329.7902409879</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="46" t="n">
+      <c r="A24" s="32" t="n">
         <v>0.9</v>
       </c>
-      <c r="B24" s="36" t="n">
+      <c r="B24" s="38" t="n">
         <f aca="false">$A24*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-B$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>37677.310655248</v>
       </c>
-      <c r="C24" s="36" t="n">
+      <c r="C24" s="38" t="n">
         <f aca="false">$A24*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-C$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>34742.5864967138</v>
       </c>
-      <c r="D24" s="36" t="n">
+      <c r="D24" s="38" t="n">
         <f aca="false">$A24*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-D$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>31925.251304521</v>
       </c>
-      <c r="E24" s="36" t="n">
+      <c r="E24" s="38" t="n">
         <f aca="false">$A24*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-E$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>28873.1381796455</v>
       </c>
-      <c r="F24" s="36" t="n">
+      <c r="F24" s="38" t="n">
         <f aca="false">$A24*(Inputs!$B$5*(Inputs!$B$16+Inputs!$B$17))*(Inputs!$B$6/60*Inputs!$B$7-F$17)-(Inputs!$B$5*Inputs!$C$26+Inputs!$C$28+Model!$C$25)</f>
         <v>25938.4140211113</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="48" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="B26" s="48"/>
       <c r="C26" s="48"/>
@@ -4257,147 +4309,147 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="34" t="s">
-        <v>198</v>
-      </c>
-      <c r="B4" s="34" t="s">
-        <v>199</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>200</v>
+      <c r="A4" s="36" t="s">
+        <v>203</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>205</v>
       </c>
       <c r="D4" s="23" t="n">
         <v>281</v>
       </c>
-      <c r="F4" s="34" t="s">
-        <v>200</v>
-      </c>
-      <c r="G4" s="35" t="n">
+      <c r="F4" s="36" t="s">
+        <v>205</v>
+      </c>
+      <c r="G4" s="37" t="n">
         <f aca="false">SUMIF($C$4:$C$58,F4,$D$4:$D$58)</f>
         <v>3165</v>
       </c>
-      <c r="H4" s="37" t="n">
+      <c r="H4" s="39" t="n">
         <f aca="false">G4/$G$8</f>
         <v>0.315176259709221</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="34" t="s">
-        <v>201</v>
-      </c>
-      <c r="B5" s="34" t="s">
-        <v>199</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>200</v>
+      <c r="A5" s="36" t="s">
+        <v>206</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="C5" s="36" t="s">
+        <v>205</v>
       </c>
       <c r="D5" s="23" t="n">
         <v>281</v>
       </c>
-      <c r="F5" s="34" t="s">
-        <v>202</v>
-      </c>
-      <c r="G5" s="35" t="n">
+      <c r="F5" s="36" t="s">
+        <v>207</v>
+      </c>
+      <c r="G5" s="37" t="n">
         <f aca="false">SUMIF($C$4:$C$58,F5,$D$4:$D$58)</f>
         <v>1201</v>
       </c>
-      <c r="H5" s="37" t="n">
+      <c r="H5" s="39" t="n">
         <f aca="false">G5/$G$8</f>
         <v>0.119597689703246</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="34" t="s">
-        <v>203</v>
-      </c>
-      <c r="B6" s="34" t="s">
-        <v>199</v>
-      </c>
-      <c r="C6" s="34" t="s">
-        <v>200</v>
+      <c r="A6" s="36" t="s">
+        <v>208</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="C6" s="36" t="s">
+        <v>205</v>
       </c>
       <c r="D6" s="23" t="n">
         <v>277</v>
       </c>
-      <c r="F6" s="34" t="s">
-        <v>204</v>
-      </c>
-      <c r="G6" s="35" t="n">
+      <c r="F6" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="G6" s="37" t="n">
         <f aca="false">SUMIF($C$4:$C$58,F6,$D$4:$D$58)</f>
         <v>4440</v>
       </c>
-      <c r="H6" s="37" t="n">
+      <c r="H6" s="39" t="n">
         <f aca="false">G6/$G$8</f>
         <v>0.442142999402509</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="C7" s="36" t="s">
         <v>205</v>
-      </c>
-      <c r="B7" s="34" t="s">
-        <v>199</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>200</v>
       </c>
       <c r="D7" s="23" t="n">
         <v>272</v>
       </c>
-      <c r="F7" s="34" t="s">
-        <v>206</v>
-      </c>
-      <c r="G7" s="35" t="n">
+      <c r="F7" s="36" t="s">
+        <v>211</v>
+      </c>
+      <c r="G7" s="37" t="n">
         <f aca="false">SUMIF($C$4:$C$58,F7,$D$4:$D$58)</f>
         <v>1236</v>
       </c>
-      <c r="H7" s="37" t="n">
+      <c r="H7" s="39" t="n">
         <f aca="false">G7/$G$8</f>
         <v>0.123083051185023</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="s">
-        <v>207</v>
-      </c>
-      <c r="B8" s="34" t="s">
-        <v>199</v>
-      </c>
-      <c r="C8" s="34" t="s">
-        <v>200</v>
+      <c r="A8" s="36" t="s">
+        <v>212</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>205</v>
       </c>
       <c r="D8" s="23" t="n">
         <v>264</v>
       </c>
       <c r="F8" s="27" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="G8" s="49" t="n">
         <f aca="false">SUM(G4:G7)</f>
@@ -4409,700 +4461,700 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="34" t="s">
-        <v>209</v>
-      </c>
-      <c r="B9" s="34" t="s">
-        <v>199</v>
-      </c>
-      <c r="C9" s="34" t="s">
-        <v>200</v>
+      <c r="A9" s="36" t="s">
+        <v>214</v>
+      </c>
+      <c r="B9" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="C9" s="36" t="s">
+        <v>205</v>
       </c>
       <c r="D9" s="23" t="n">
         <v>263</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="34" t="s">
-        <v>210</v>
-      </c>
-      <c r="B10" s="34" t="s">
-        <v>199</v>
-      </c>
-      <c r="C10" s="34" t="s">
-        <v>200</v>
+      <c r="A10" s="36" t="s">
+        <v>215</v>
+      </c>
+      <c r="B10" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="C10" s="36" t="s">
+        <v>205</v>
       </c>
       <c r="D10" s="23" t="n">
         <v>252</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34" t="s">
-        <v>211</v>
-      </c>
-      <c r="B11" s="34" t="s">
-        <v>199</v>
-      </c>
-      <c r="C11" s="34" t="s">
-        <v>200</v>
+      <c r="A11" s="36" t="s">
+        <v>216</v>
+      </c>
+      <c r="B11" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="36" t="s">
+        <v>205</v>
       </c>
       <c r="D11" s="23" t="n">
         <v>249</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34" t="s">
-        <v>212</v>
-      </c>
-      <c r="B12" s="34" t="s">
-        <v>213</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>200</v>
+      <c r="A12" s="36" t="s">
+        <v>217</v>
+      </c>
+      <c r="B12" s="36" t="s">
+        <v>218</v>
+      </c>
+      <c r="C12" s="36" t="s">
+        <v>205</v>
       </c>
       <c r="D12" s="23" t="n">
         <v>266</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34" t="s">
-        <v>214</v>
-      </c>
-      <c r="B13" s="34" t="s">
-        <v>213</v>
-      </c>
-      <c r="C13" s="34" t="s">
-        <v>200</v>
+      <c r="A13" s="36" t="s">
+        <v>219</v>
+      </c>
+      <c r="B13" s="36" t="s">
+        <v>218</v>
+      </c>
+      <c r="C13" s="36" t="s">
+        <v>205</v>
       </c>
       <c r="D13" s="23" t="n">
         <v>259</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34" t="s">
-        <v>215</v>
-      </c>
-      <c r="B14" s="34" t="s">
-        <v>213</v>
-      </c>
-      <c r="C14" s="34" t="s">
-        <v>200</v>
+      <c r="A14" s="36" t="s">
+        <v>220</v>
+      </c>
+      <c r="B14" s="36" t="s">
+        <v>218</v>
+      </c>
+      <c r="C14" s="36" t="s">
+        <v>205</v>
       </c>
       <c r="D14" s="23" t="n">
         <v>251</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34" t="s">
-        <v>216</v>
-      </c>
-      <c r="B15" s="34" t="s">
-        <v>213</v>
-      </c>
-      <c r="C15" s="34" t="s">
-        <v>200</v>
+      <c r="A15" s="36" t="s">
+        <v>221</v>
+      </c>
+      <c r="B15" s="36" t="s">
+        <v>218</v>
+      </c>
+      <c r="C15" s="36" t="s">
+        <v>205</v>
       </c>
       <c r="D15" s="23" t="n">
         <v>250</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34" t="s">
-        <v>217</v>
-      </c>
-      <c r="B16" s="34" t="s">
-        <v>218</v>
-      </c>
-      <c r="C16" s="34" t="s">
-        <v>202</v>
+      <c r="A16" s="36" t="s">
+        <v>222</v>
+      </c>
+      <c r="B16" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="C16" s="36" t="s">
+        <v>207</v>
       </c>
       <c r="D16" s="23" t="n">
         <v>361</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="34" t="s">
-        <v>219</v>
-      </c>
-      <c r="B17" s="34" t="s">
-        <v>220</v>
-      </c>
-      <c r="C17" s="34" t="s">
-        <v>202</v>
+      <c r="A17" s="36" t="s">
+        <v>224</v>
+      </c>
+      <c r="B17" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="C17" s="36" t="s">
+        <v>207</v>
       </c>
       <c r="D17" s="23" t="n">
         <v>179</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="34" t="s">
-        <v>221</v>
-      </c>
-      <c r="B18" s="34" t="s">
-        <v>222</v>
-      </c>
-      <c r="C18" s="34" t="s">
-        <v>202</v>
+      <c r="A18" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="B18" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="C18" s="36" t="s">
+        <v>207</v>
       </c>
       <c r="D18" s="23" t="n">
         <v>268</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="34" t="s">
-        <v>223</v>
-      </c>
-      <c r="B19" s="34" t="s">
-        <v>224</v>
-      </c>
-      <c r="C19" s="34" t="s">
-        <v>202</v>
+      <c r="A19" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="B19" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="C19" s="36" t="s">
+        <v>207</v>
       </c>
       <c r="D19" s="23" t="n">
         <v>185</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34" t="s">
-        <v>225</v>
-      </c>
-      <c r="B20" s="34" t="s">
-        <v>224</v>
-      </c>
-      <c r="C20" s="34" t="s">
-        <v>202</v>
+      <c r="A20" s="36" t="s">
+        <v>230</v>
+      </c>
+      <c r="B20" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="C20" s="36" t="s">
+        <v>207</v>
       </c>
       <c r="D20" s="23" t="n">
         <v>178</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="34" t="s">
-        <v>226</v>
-      </c>
-      <c r="B21" s="34" t="s">
-        <v>224</v>
-      </c>
-      <c r="C21" s="34" t="s">
-        <v>202</v>
+      <c r="A21" s="36" t="s">
+        <v>231</v>
+      </c>
+      <c r="B21" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="C21" s="36" t="s">
+        <v>207</v>
       </c>
       <c r="D21" s="23" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="34" t="s">
-        <v>227</v>
-      </c>
-      <c r="B22" s="34" t="s">
-        <v>228</v>
-      </c>
-      <c r="C22" s="34" t="s">
-        <v>204</v>
+      <c r="A22" s="36" t="s">
+        <v>232</v>
+      </c>
+      <c r="B22" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="C22" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D22" s="23" t="n">
         <v>153</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="34" t="s">
-        <v>229</v>
-      </c>
-      <c r="B23" s="34" t="s">
-        <v>228</v>
-      </c>
-      <c r="C23" s="34" t="s">
-        <v>204</v>
+      <c r="A23" s="36" t="s">
+        <v>234</v>
+      </c>
+      <c r="B23" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="C23" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D23" s="23" t="n">
         <v>129</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="34" t="s">
-        <v>230</v>
-      </c>
-      <c r="B24" s="34" t="s">
-        <v>228</v>
-      </c>
-      <c r="C24" s="34" t="s">
-        <v>204</v>
+      <c r="A24" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="B24" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="C24" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D24" s="23" t="n">
         <v>114</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="34" t="s">
-        <v>231</v>
-      </c>
-      <c r="B25" s="34" t="s">
-        <v>228</v>
-      </c>
-      <c r="C25" s="34" t="s">
-        <v>204</v>
+      <c r="A25" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="B25" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="C25" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D25" s="23" t="n">
         <v>51</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="34" t="s">
-        <v>232</v>
-      </c>
-      <c r="B26" s="34" t="s">
-        <v>228</v>
-      </c>
-      <c r="C26" s="34" t="s">
-        <v>204</v>
+      <c r="A26" s="36" t="s">
+        <v>237</v>
+      </c>
+      <c r="B26" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="C26" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D26" s="23" t="n">
         <v>51</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="34" t="s">
+      <c r="A27" s="36" t="s">
+        <v>238</v>
+      </c>
+      <c r="B27" s="36" t="s">
         <v>233</v>
       </c>
-      <c r="B27" s="34" t="s">
-        <v>228</v>
-      </c>
-      <c r="C27" s="34" t="s">
-        <v>204</v>
+      <c r="C27" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D27" s="23" t="n">
         <v>48</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="34" t="s">
-        <v>234</v>
-      </c>
-      <c r="B28" s="34" t="s">
-        <v>228</v>
-      </c>
-      <c r="C28" s="34" t="s">
-        <v>204</v>
+      <c r="A28" s="36" t="s">
+        <v>239</v>
+      </c>
+      <c r="B28" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="C28" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D28" s="23" t="n">
         <v>36</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="34" t="s">
-        <v>235</v>
-      </c>
-      <c r="B29" s="34" t="s">
-        <v>236</v>
-      </c>
-      <c r="C29" s="34" t="s">
-        <v>204</v>
+      <c r="A29" s="36" t="s">
+        <v>240</v>
+      </c>
+      <c r="B29" s="36" t="s">
+        <v>241</v>
+      </c>
+      <c r="C29" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D29" s="23" t="n">
         <v>135</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="34" t="s">
-        <v>237</v>
-      </c>
-      <c r="B30" s="34" t="s">
-        <v>236</v>
-      </c>
-      <c r="C30" s="34" t="s">
-        <v>204</v>
+      <c r="A30" s="36" t="s">
+        <v>242</v>
+      </c>
+      <c r="B30" s="36" t="s">
+        <v>241</v>
+      </c>
+      <c r="C30" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D30" s="23" t="n">
         <v>134</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="34" t="s">
-        <v>238</v>
-      </c>
-      <c r="B31" s="34" t="s">
-        <v>236</v>
-      </c>
-      <c r="C31" s="34" t="s">
-        <v>204</v>
+      <c r="A31" s="36" t="s">
+        <v>243</v>
+      </c>
+      <c r="B31" s="36" t="s">
+        <v>241</v>
+      </c>
+      <c r="C31" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D31" s="23" t="n">
         <v>134</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="34" t="s">
-        <v>239</v>
-      </c>
-      <c r="B32" s="34" t="s">
-        <v>236</v>
-      </c>
-      <c r="C32" s="34" t="s">
-        <v>204</v>
+      <c r="A32" s="36" t="s">
+        <v>244</v>
+      </c>
+      <c r="B32" s="36" t="s">
+        <v>241</v>
+      </c>
+      <c r="C32" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D32" s="23" t="n">
         <v>130</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="34" t="s">
-        <v>240</v>
-      </c>
-      <c r="B33" s="34" t="s">
-        <v>236</v>
-      </c>
-      <c r="C33" s="34" t="s">
-        <v>204</v>
+      <c r="A33" s="36" t="s">
+        <v>245</v>
+      </c>
+      <c r="B33" s="36" t="s">
+        <v>241</v>
+      </c>
+      <c r="C33" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D33" s="23" t="n">
         <v>125</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="34" t="s">
+      <c r="A34" s="36" t="s">
+        <v>246</v>
+      </c>
+      <c r="B34" s="36" t="s">
         <v>241</v>
       </c>
-      <c r="B34" s="34" t="s">
-        <v>236</v>
-      </c>
-      <c r="C34" s="34" t="s">
-        <v>204</v>
+      <c r="C34" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D34" s="23" t="n">
         <v>123</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="34" t="s">
-        <v>242</v>
-      </c>
-      <c r="B35" s="34" t="s">
-        <v>236</v>
-      </c>
-      <c r="C35" s="34" t="s">
-        <v>204</v>
+      <c r="A35" s="36" t="s">
+        <v>247</v>
+      </c>
+      <c r="B35" s="36" t="s">
+        <v>241</v>
+      </c>
+      <c r="C35" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D35" s="23" t="n">
         <v>117</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="34" t="s">
-        <v>243</v>
-      </c>
-      <c r="B36" s="34" t="s">
-        <v>244</v>
-      </c>
-      <c r="C36" s="34" t="s">
-        <v>204</v>
+      <c r="A36" s="36" t="s">
+        <v>248</v>
+      </c>
+      <c r="B36" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="C36" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D36" s="23" t="n">
         <v>149</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="34" t="s">
-        <v>245</v>
-      </c>
-      <c r="B37" s="34" t="s">
-        <v>244</v>
-      </c>
-      <c r="C37" s="34" t="s">
-        <v>204</v>
+      <c r="A37" s="36" t="s">
+        <v>250</v>
+      </c>
+      <c r="B37" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="C37" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D37" s="23" t="n">
         <v>140</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="34" t="s">
-        <v>246</v>
-      </c>
-      <c r="B38" s="34" t="s">
-        <v>244</v>
-      </c>
-      <c r="C38" s="34" t="s">
-        <v>204</v>
+      <c r="A38" s="36" t="s">
+        <v>251</v>
+      </c>
+      <c r="B38" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="C38" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D38" s="23" t="n">
         <v>139</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="34" t="s">
-        <v>247</v>
-      </c>
-      <c r="B39" s="34" t="s">
-        <v>244</v>
-      </c>
-      <c r="C39" s="34" t="s">
-        <v>204</v>
+      <c r="A39" s="36" t="s">
+        <v>252</v>
+      </c>
+      <c r="B39" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="C39" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D39" s="23" t="n">
         <v>133</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="34" t="s">
-        <v>248</v>
-      </c>
-      <c r="B40" s="34" t="s">
-        <v>244</v>
-      </c>
-      <c r="C40" s="34" t="s">
-        <v>204</v>
+      <c r="A40" s="36" t="s">
+        <v>253</v>
+      </c>
+      <c r="B40" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="C40" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D40" s="23" t="n">
         <v>127</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="34" t="s">
+      <c r="A41" s="36" t="s">
+        <v>254</v>
+      </c>
+      <c r="B41" s="36" t="s">
         <v>249</v>
       </c>
-      <c r="B41" s="34" t="s">
-        <v>244</v>
-      </c>
-      <c r="C41" s="34" t="s">
-        <v>204</v>
+      <c r="C41" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D41" s="23" t="n">
         <v>112</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="34" t="s">
-        <v>250</v>
-      </c>
-      <c r="B42" s="34" t="s">
-        <v>220</v>
-      </c>
-      <c r="C42" s="34" t="s">
-        <v>204</v>
+      <c r="A42" s="36" t="s">
+        <v>255</v>
+      </c>
+      <c r="B42" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="C42" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D42" s="23" t="n">
         <v>191</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="34" t="s">
-        <v>251</v>
-      </c>
-      <c r="B43" s="34" t="s">
-        <v>220</v>
-      </c>
-      <c r="C43" s="34" t="s">
-        <v>204</v>
+      <c r="A43" s="36" t="s">
+        <v>256</v>
+      </c>
+      <c r="B43" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="C43" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D43" s="23" t="n">
         <v>180</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="34" t="s">
-        <v>252</v>
-      </c>
-      <c r="B44" s="34" t="s">
-        <v>220</v>
-      </c>
-      <c r="C44" s="34" t="s">
-        <v>204</v>
+      <c r="A44" s="36" t="s">
+        <v>257</v>
+      </c>
+      <c r="B44" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="C44" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D44" s="23" t="n">
         <v>177</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="34" t="s">
-        <v>253</v>
-      </c>
-      <c r="B45" s="34" t="s">
-        <v>220</v>
-      </c>
-      <c r="C45" s="34" t="s">
-        <v>204</v>
+      <c r="A45" s="36" t="s">
+        <v>258</v>
+      </c>
+      <c r="B45" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="C45" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D45" s="23" t="n">
         <v>176</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="34" t="s">
-        <v>254</v>
-      </c>
-      <c r="B46" s="34" t="s">
-        <v>220</v>
-      </c>
-      <c r="C46" s="34" t="s">
-        <v>204</v>
+      <c r="A46" s="36" t="s">
+        <v>259</v>
+      </c>
+      <c r="B46" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="C46" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D46" s="23" t="n">
         <v>167</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="34" t="s">
-        <v>255</v>
-      </c>
-      <c r="B47" s="34" t="s">
-        <v>222</v>
-      </c>
-      <c r="C47" s="34" t="s">
-        <v>204</v>
+      <c r="A47" s="36" t="s">
+        <v>260</v>
+      </c>
+      <c r="B47" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="C47" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D47" s="23" t="n">
         <v>261</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="34" t="s">
-        <v>256</v>
-      </c>
-      <c r="B48" s="34" t="s">
-        <v>222</v>
-      </c>
-      <c r="C48" s="34" t="s">
-        <v>204</v>
+      <c r="A48" s="36" t="s">
+        <v>261</v>
+      </c>
+      <c r="B48" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="C48" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D48" s="23" t="n">
         <v>248</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="34" t="s">
-        <v>257</v>
-      </c>
-      <c r="B49" s="34" t="s">
-        <v>222</v>
-      </c>
-      <c r="C49" s="34" t="s">
-        <v>204</v>
+      <c r="A49" s="36" t="s">
+        <v>262</v>
+      </c>
+      <c r="B49" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="C49" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D49" s="23" t="n">
         <v>243</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="34" t="s">
-        <v>258</v>
-      </c>
-      <c r="B50" s="34" t="s">
-        <v>224</v>
-      </c>
-      <c r="C50" s="34" t="s">
-        <v>204</v>
+      <c r="A50" s="36" t="s">
+        <v>263</v>
+      </c>
+      <c r="B50" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="C50" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D50" s="23" t="n">
         <v>190</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="34" t="s">
-        <v>259</v>
-      </c>
-      <c r="B51" s="34" t="s">
-        <v>224</v>
-      </c>
-      <c r="C51" s="34" t="s">
-        <v>204</v>
+      <c r="A51" s="36" t="s">
+        <v>264</v>
+      </c>
+      <c r="B51" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="C51" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D51" s="23" t="n">
         <v>165</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="B52" s="34" t="s">
-        <v>224</v>
-      </c>
-      <c r="C52" s="34" t="s">
-        <v>204</v>
+      <c r="A52" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="B52" s="36" t="s">
+        <v>229</v>
+      </c>
+      <c r="C52" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="D52" s="23" t="n">
         <v>162</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="34" t="s">
-        <v>261</v>
-      </c>
-      <c r="B53" s="34" t="s">
-        <v>218</v>
-      </c>
-      <c r="C53" s="34" t="s">
-        <v>206</v>
+      <c r="A53" s="36" t="s">
+        <v>266</v>
+      </c>
+      <c r="B53" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="C53" s="36" t="s">
+        <v>211</v>
       </c>
       <c r="D53" s="23" t="n">
         <v>351</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="34" t="s">
-        <v>262</v>
-      </c>
-      <c r="B54" s="34" t="s">
-        <v>218</v>
-      </c>
-      <c r="C54" s="34" t="s">
-        <v>206</v>
+      <c r="A54" s="36" t="s">
+        <v>267</v>
+      </c>
+      <c r="B54" s="36" t="s">
+        <v>223</v>
+      </c>
+      <c r="C54" s="36" t="s">
+        <v>211</v>
       </c>
       <c r="D54" s="23" t="n">
         <v>336</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="34" t="s">
-        <v>263</v>
-      </c>
-      <c r="B55" s="34" t="s">
-        <v>228</v>
-      </c>
-      <c r="C55" s="34" t="s">
-        <v>206</v>
+      <c r="A55" s="36" t="s">
+        <v>268</v>
+      </c>
+      <c r="B55" s="36" t="s">
+        <v>233</v>
+      </c>
+      <c r="C55" s="36" t="s">
+        <v>211</v>
       </c>
       <c r="D55" s="23" t="n">
         <v>131</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="34" t="s">
-        <v>264</v>
-      </c>
-      <c r="B56" s="34" t="s">
-        <v>236</v>
-      </c>
-      <c r="C56" s="34" t="s">
-        <v>206</v>
+      <c r="A56" s="36" t="s">
+        <v>269</v>
+      </c>
+      <c r="B56" s="36" t="s">
+        <v>241</v>
+      </c>
+      <c r="C56" s="36" t="s">
+        <v>211</v>
       </c>
       <c r="D56" s="23" t="n">
         <v>142</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="34" t="s">
-        <v>265</v>
-      </c>
-      <c r="B57" s="34" t="s">
-        <v>244</v>
-      </c>
-      <c r="C57" s="34" t="s">
-        <v>206</v>
+      <c r="A57" s="36" t="s">
+        <v>270</v>
+      </c>
+      <c r="B57" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="C57" s="36" t="s">
+        <v>211</v>
       </c>
       <c r="D57" s="23" t="n">
         <v>139</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="34" t="s">
-        <v>266</v>
-      </c>
-      <c r="B58" s="34" t="s">
-        <v>244</v>
-      </c>
-      <c r="C58" s="34" t="s">
-        <v>206</v>
+      <c r="A58" s="36" t="s">
+        <v>271</v>
+      </c>
+      <c r="B58" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="C58" s="36" t="s">
+        <v>211</v>
       </c>
       <c r="D58" s="23" t="n">
         <v>137</v>
@@ -5110,7 +5162,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="27" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="D59" s="49" t="n">
         <f aca="false">SUM(D4:D58)</f>
@@ -5119,7 +5171,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>

</xml_diff>